<commit_message>
feat: stamp Invoice/PL PDFs and correct PF packing-list weights
PF packing lists now number cartons and scale N/W G/W from PO totals, falling back to DATA BASE per carton with matching source tracing. Invoice/PL PDFs overlay seller stamps after LibreOffice conversion without blocking export when a chop file is missing.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/customer_profiles/pf/templates/gs/invoice.xlsx
+++ b/customer_profiles/pf/templates/gs/invoice.xlsx
@@ -1140,7 +1140,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="133">
+  <cellXfs count="146">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1533,6 +1533,45 @@
     </xf>
     <xf numFmtId="168" fontId="18" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="76">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="75">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="75">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="57">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="56">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="75">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="76">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="77">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="87">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="87">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="1" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="117">
@@ -2263,6 +2302,7 @@
       <c r="B20" s="1" t="n"/>
       <c r="C20" s="1" t="n"/>
       <c r="D20" s="1" t="n"/>
+      <c r="E20" s="133" t="n"/>
       <c r="F20" s="126" t="n"/>
       <c r="G20" s="127" t="n"/>
       <c r="H20" s="128" t="n"/>
@@ -2272,6 +2312,7 @@
       <c r="B21" s="65" t="n"/>
       <c r="C21" s="65" t="n"/>
       <c r="D21" s="65" t="n"/>
+      <c r="E21" s="133" t="n"/>
       <c r="F21" s="129" t="inlineStr">
         <is>
           <t xml:space="preserve">Sub-Total </t>
@@ -2320,56 +2361,61 @@
       <c r="H25" s="74" t="n"/>
       <c r="I25" s="32" t="n"/>
     </row>
-    <row r="26"/>
     <row r="27" ht="11.64999961853027" customHeight="1" s="123"/>
     <row r="28" ht="21" customFormat="1" customHeight="1" s="5">
       <c r="B28" s="131" t="n"/>
     </row>
     <row r="29" ht="27.75" customFormat="1" customHeight="1" s="5">
-      <c r="A29" s="76" t="inlineStr">
+      <c r="A29" s="134" t="inlineStr">
         <is>
           <t>Cost breakdown and actual manufacturer breakdown (Additional info required for NA specified product)</t>
         </is>
       </c>
-      <c r="B29" s="76" t="n"/>
-      <c r="D29" s="77" t="n"/>
-      <c r="E29" s="77" t="n"/>
-      <c r="G29" s="78" t="n"/>
-      <c r="H29" s="78" t="n"/>
+      <c r="B29" s="135" t="n"/>
+      <c r="C29" s="136" t="n"/>
+      <c r="D29" s="137" t="n"/>
+      <c r="E29" s="137" t="n"/>
+      <c r="F29" s="136" t="n"/>
+      <c r="G29" s="138" t="n"/>
+      <c r="H29" s="138" t="n"/>
       <c r="I29" s="79" t="n"/>
       <c r="J29" s="79" t="n"/>
     </row>
     <row r="30" ht="16.5" customFormat="1" customHeight="1" s="5">
-      <c r="A30" s="80" t="n"/>
-      <c r="B30" s="81" t="inlineStr">
+      <c r="A30" s="139" t="n"/>
+      <c r="B30" s="60" t="inlineStr">
         <is>
           <t>PO Number</t>
         </is>
       </c>
-      <c r="C30" s="81" t="inlineStr">
+      <c r="C30" s="60" t="inlineStr">
         <is>
           <t>PO item Line Number</t>
         </is>
       </c>
-      <c r="D30" s="82" t="inlineStr">
+      <c r="D30" s="140" t="inlineStr">
         <is>
           <t>Item Number</t>
         </is>
       </c>
-      <c r="E30" s="83" t="inlineStr">
+      <c r="E30" s="141" t="inlineStr">
         <is>
           <t xml:space="preserve">Description </t>
         </is>
       </c>
-      <c r="F30" s="132" t="inlineStr">
+      <c r="F30" s="124" t="inlineStr">
         <is>
           <t>USD unit price breakdown</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="85" t="n"/>
-      <c r="B31" s="85" t="n"/>
+    <row r="31" ht="15.94999980926514" customHeight="1" s="123">
+      <c r="A31" s="142" t="n"/>
+      <c r="B31" s="143" t="n"/>
+      <c r="C31" s="144" t="n"/>
+      <c r="D31" s="144" t="n"/>
+      <c r="E31" s="144" t="n"/>
+      <c r="F31" s="145" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>